<commit_message>
update asa approval date and rerun pipeline
</commit_message>
<xml_diff>
--- a/inst/extdata/region/2026-08-10/wb_projects_gov_afw.xlsx
+++ b/inst/extdata/region/2026-08-10/wb_projects_gov_afw.xlsx
@@ -2063,9 +2063,11 @@
         <v>40</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2025</v>
-      </c>
-      <c r="H2" s="2"/>
+        <v>2024</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>45269</v>
+      </c>
       <c r="I2" s="2" t="s">
         <v>133</v>
       </c>

</xml_diff>